<commit_message>
done with Nov import
</commit_message>
<xml_diff>
--- a/import/importFile-Sample.xlsx
+++ b/import/importFile-Sample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\projects\resorts\repo\avrlodge_v2\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27085A56-0EA7-4CFA-9D43-4C3E2E2D159F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFBA8AA-BAC3-4D2E-96BE-D01A7AE158DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{61EC7E60-39E1-4E22-9A23-5C6CFCE41CF9}"/>
   </bookViews>
@@ -2486,7 +2486,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Deepika  (Trans
+          <t xml:space="preserve">Deepika
 </t>
         </r>
         <r>
@@ -6099,22 +6099,46 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6123,6 +6147,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -6138,39 +6171,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6680,22 +6680,24 @@
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A3" s="32">
+      <c r="A3" s="21">
         <v>101</v>
       </c>
       <c r="B3" s="6">
         <v>6</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="8">
+        <v>2</v>
+      </c>
       <c r="E3" s="7">
         <v>6</v>
       </c>
       <c r="F3" s="7">
         <v>6</v>
       </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="25"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="14"/>
       <c r="J3" s="7">
         <v>6</v>
       </c>
@@ -6764,24 +6766,24 @@
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A4" s="32">
+      <c r="A4" s="21">
         <v>102</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="26">
         <v>4</v>
       </c>
       <c r="C4" s="8">
         <v>4</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>2</v>
       </c>
       <c r="F4" s="7">
         <v>4</v>
       </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="28"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="17"/>
       <c r="J4" s="7">
         <v>4</v>
       </c>
@@ -6839,7 +6841,7 @@
       <c r="AB4" s="7">
         <v>4</v>
       </c>
-      <c r="AC4" s="9">
+      <c r="AC4" s="26">
         <v>4</v>
       </c>
       <c r="AD4" s="6">
@@ -6850,170 +6852,174 @@
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A5" s="32">
+      <c r="A5" s="21">
         <v>103</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="8">
         <v>2</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="12">
-        <v>2</v>
-      </c>
-      <c r="F5" s="10">
-        <v>2</v>
-      </c>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="10">
-        <v>2</v>
-      </c>
-      <c r="K5" s="10">
-        <v>2</v>
-      </c>
-      <c r="L5" s="12">
-        <v>2</v>
-      </c>
-      <c r="M5" s="12">
-        <v>2</v>
-      </c>
-      <c r="N5" s="10">
-        <v>2</v>
-      </c>
-      <c r="P5" s="10">
-        <v>2</v>
-      </c>
-      <c r="Q5" s="12">
-        <v>2</v>
-      </c>
-      <c r="R5" s="12">
-        <v>2</v>
-      </c>
-      <c r="S5" s="12">
-        <v>2</v>
-      </c>
-      <c r="T5" s="10">
-        <v>2</v>
-      </c>
-      <c r="U5" s="12">
-        <v>2</v>
-      </c>
-      <c r="V5" s="12">
-        <v>2</v>
-      </c>
-      <c r="W5" s="10">
-        <v>2</v>
-      </c>
-      <c r="X5" s="10">
-        <v>2</v>
-      </c>
-      <c r="Y5" s="10">
-        <v>2</v>
-      </c>
-      <c r="Z5" s="10">
-        <v>2</v>
-      </c>
-      <c r="AA5" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB5" s="10">
-        <v>2</v>
-      </c>
-      <c r="AC5" s="11"/>
-      <c r="AD5" s="10">
-        <v>2</v>
-      </c>
-      <c r="AE5" s="10">
+      <c r="D5" s="11">
+        <v>2</v>
+      </c>
+      <c r="E5" s="10">
+        <v>2</v>
+      </c>
+      <c r="F5" s="9">
+        <v>2</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="9">
+        <v>2</v>
+      </c>
+      <c r="K5" s="9">
+        <v>2</v>
+      </c>
+      <c r="L5" s="10">
+        <v>2</v>
+      </c>
+      <c r="M5" s="10">
+        <v>2</v>
+      </c>
+      <c r="N5" s="9">
+        <v>2</v>
+      </c>
+      <c r="P5" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="10">
+        <v>2</v>
+      </c>
+      <c r="R5" s="10">
+        <v>2</v>
+      </c>
+      <c r="S5" s="10">
+        <v>2</v>
+      </c>
+      <c r="T5" s="9">
+        <v>2</v>
+      </c>
+      <c r="U5" s="10">
+        <v>2</v>
+      </c>
+      <c r="V5" s="10">
+        <v>2</v>
+      </c>
+      <c r="W5" s="9">
+        <v>2</v>
+      </c>
+      <c r="X5" s="9">
+        <v>2</v>
+      </c>
+      <c r="Y5" s="9">
+        <v>2</v>
+      </c>
+      <c r="Z5" s="9">
+        <v>2</v>
+      </c>
+      <c r="AA5" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB5" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC5" s="28"/>
+      <c r="AD5" s="9">
+        <v>2</v>
+      </c>
+      <c r="AE5" s="9">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A6" s="32">
+      <c r="A6" s="21">
         <v>104</v>
       </c>
-      <c r="B6" s="11"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="10">
-        <v>2</v>
-      </c>
-      <c r="F6" s="10">
-        <v>2</v>
-      </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="10">
-        <v>2</v>
-      </c>
-      <c r="K6" s="10">
-        <v>2</v>
-      </c>
-      <c r="L6" s="10">
-        <v>2</v>
-      </c>
-      <c r="M6" s="10">
-        <v>2</v>
-      </c>
-      <c r="N6" s="10">
-        <v>2</v>
-      </c>
-      <c r="O6" s="10">
-        <v>2</v>
-      </c>
-      <c r="P6" s="10">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="10">
-        <v>2</v>
-      </c>
-      <c r="R6" s="12">
-        <v>2</v>
-      </c>
-      <c r="S6" s="10">
-        <v>2</v>
-      </c>
-      <c r="T6" s="10">
-        <v>2</v>
-      </c>
-      <c r="U6" s="12">
-        <v>2</v>
-      </c>
-      <c r="V6" s="10">
-        <v>2</v>
-      </c>
-      <c r="W6" s="10">
-        <v>2</v>
-      </c>
-      <c r="X6" s="10">
-        <v>2</v>
-      </c>
-      <c r="Y6" s="12">
-        <v>2</v>
-      </c>
-      <c r="Z6" s="10">
-        <v>2</v>
-      </c>
-      <c r="AA6" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB6" s="12">
-        <v>2</v>
-      </c>
-      <c r="AC6" s="12">
-        <v>2</v>
-      </c>
-      <c r="AD6" s="12">
-        <v>2</v>
-      </c>
-      <c r="AE6" s="10">
+      <c r="D6" s="11">
+        <v>4</v>
+      </c>
+      <c r="E6" s="9">
+        <v>2</v>
+      </c>
+      <c r="F6" s="9">
+        <v>2</v>
+      </c>
+      <c r="G6" s="15"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="9">
+        <v>2</v>
+      </c>
+      <c r="K6" s="9">
+        <v>2</v>
+      </c>
+      <c r="L6" s="9">
+        <v>2</v>
+      </c>
+      <c r="M6" s="9">
+        <v>2</v>
+      </c>
+      <c r="N6" s="9">
+        <v>2</v>
+      </c>
+      <c r="O6" s="9">
+        <v>2</v>
+      </c>
+      <c r="P6" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="9">
+        <v>2</v>
+      </c>
+      <c r="R6" s="10">
+        <v>2</v>
+      </c>
+      <c r="S6" s="9">
+        <v>2</v>
+      </c>
+      <c r="T6" s="9">
+        <v>2</v>
+      </c>
+      <c r="U6" s="10">
+        <v>2</v>
+      </c>
+      <c r="V6" s="9">
+        <v>2</v>
+      </c>
+      <c r="W6" s="9">
+        <v>2</v>
+      </c>
+      <c r="X6" s="9">
+        <v>2</v>
+      </c>
+      <c r="Y6" s="10">
+        <v>2</v>
+      </c>
+      <c r="Z6" s="9">
+        <v>2</v>
+      </c>
+      <c r="AA6" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB6" s="10">
+        <v>2</v>
+      </c>
+      <c r="AC6" s="10">
+        <v>2</v>
+      </c>
+      <c r="AD6" s="10">
+        <v>2</v>
+      </c>
+      <c r="AE6" s="9">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A7" s="32">
+      <c r="A7" s="21">
         <v>105</v>
       </c>
       <c r="B7" s="6">
@@ -7026,9 +7032,9 @@
       <c r="F7" s="7">
         <v>4</v>
       </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="17"/>
       <c r="J7" s="6">
         <v>4</v>
       </c>
@@ -7097,242 +7103,246 @@
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A8" s="32">
+      <c r="A8" s="21">
         <v>106</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="10">
         <v>6</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="E8" s="10">
+      <c r="E8" s="9">
         <v>6</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="9">
         <v>6</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="10">
+      <c r="G8" s="15"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="9">
         <v>6</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="9">
         <v>6</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="9">
         <v>6</v>
       </c>
-      <c r="M8" s="12">
+      <c r="M8" s="10">
         <v>6</v>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="10">
         <v>6</v>
       </c>
-      <c r="O8" s="15">
+      <c r="O8" s="23">
         <v>6</v>
       </c>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="10">
+      <c r="P8" s="24"/>
+      <c r="Q8" s="9">
         <v>6</v>
       </c>
-      <c r="R8" s="10">
+      <c r="R8" s="9">
         <v>6</v>
       </c>
-      <c r="S8" s="10">
+      <c r="S8" s="9">
         <v>6</v>
       </c>
-      <c r="T8" s="10">
+      <c r="T8" s="9">
         <v>6</v>
       </c>
-      <c r="U8" s="10">
+      <c r="U8" s="9">
         <v>6</v>
       </c>
-      <c r="V8" s="10">
+      <c r="V8" s="9">
         <v>6</v>
       </c>
-      <c r="W8" s="10">
+      <c r="W8" s="9">
         <v>6</v>
       </c>
-      <c r="X8" s="10">
+      <c r="X8" s="9">
         <v>6</v>
       </c>
-      <c r="Y8" s="10">
+      <c r="Y8" s="9">
         <v>6</v>
       </c>
-      <c r="Z8" s="12">
+      <c r="Z8" s="10">
         <v>6</v>
       </c>
-      <c r="AA8" s="10">
+      <c r="AA8" s="9">
         <v>6</v>
       </c>
-      <c r="AB8" s="10">
+      <c r="AB8" s="9">
         <v>6</v>
       </c>
-      <c r="AC8" s="10">
+      <c r="AC8" s="9">
         <v>6</v>
       </c>
-      <c r="AD8" s="10">
+      <c r="AD8" s="9">
         <v>6</v>
       </c>
-      <c r="AE8" s="10">
+      <c r="AE8" s="9">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A9" s="33">
+      <c r="A9" s="22">
         <v>107</v>
       </c>
-      <c r="B9" s="17"/>
+      <c r="B9" s="25">
+        <v>2</v>
+      </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="10">
-        <v>2</v>
-      </c>
-      <c r="F9" s="12">
-        <v>2</v>
-      </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="10">
-        <v>2</v>
-      </c>
-      <c r="K9" s="10">
-        <v>2</v>
-      </c>
-      <c r="L9" s="10">
-        <v>2</v>
-      </c>
-      <c r="M9" s="10">
-        <v>2</v>
-      </c>
-      <c r="N9" s="10">
-        <v>2</v>
-      </c>
-      <c r="O9" s="12">
-        <v>2</v>
-      </c>
-      <c r="P9" s="12">
-        <v>2</v>
-      </c>
-      <c r="Q9" s="10">
-        <v>2</v>
-      </c>
-      <c r="R9" s="10">
-        <v>2</v>
-      </c>
-      <c r="S9" s="12">
-        <v>2</v>
-      </c>
-      <c r="T9" s="12">
-        <v>2</v>
-      </c>
-      <c r="U9" s="12">
-        <v>2</v>
-      </c>
-      <c r="V9" s="15">
-        <v>2</v>
-      </c>
-      <c r="W9" s="16"/>
-      <c r="X9" s="10">
-        <v>2</v>
-      </c>
-      <c r="Y9" s="12">
-        <v>2</v>
-      </c>
-      <c r="Z9" s="12">
-        <v>2</v>
-      </c>
-      <c r="AA9" s="10">
-        <v>2</v>
-      </c>
-      <c r="AB9" s="10">
-        <v>2</v>
-      </c>
-      <c r="AC9" s="19">
-        <v>2</v>
-      </c>
-      <c r="AD9" s="20"/>
-      <c r="AE9" s="10">
+      <c r="D9" s="29">
+        <v>2</v>
+      </c>
+      <c r="E9" s="9">
+        <v>2</v>
+      </c>
+      <c r="F9" s="10">
+        <v>2</v>
+      </c>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="9">
+        <v>2</v>
+      </c>
+      <c r="K9" s="9">
+        <v>2</v>
+      </c>
+      <c r="L9" s="9">
+        <v>2</v>
+      </c>
+      <c r="M9" s="9">
+        <v>2</v>
+      </c>
+      <c r="N9" s="9">
+        <v>2</v>
+      </c>
+      <c r="O9" s="10">
+        <v>2</v>
+      </c>
+      <c r="P9" s="10">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="9">
+        <v>2</v>
+      </c>
+      <c r="R9" s="9">
+        <v>2</v>
+      </c>
+      <c r="S9" s="10">
+        <v>2</v>
+      </c>
+      <c r="T9" s="10">
+        <v>2</v>
+      </c>
+      <c r="U9" s="10">
+        <v>2</v>
+      </c>
+      <c r="V9" s="23">
+        <v>2</v>
+      </c>
+      <c r="W9" s="24"/>
+      <c r="X9" s="9">
+        <v>2</v>
+      </c>
+      <c r="Y9" s="10">
+        <v>2</v>
+      </c>
+      <c r="Z9" s="10">
+        <v>2</v>
+      </c>
+      <c r="AA9" s="9">
+        <v>2</v>
+      </c>
+      <c r="AB9" s="9">
+        <v>2</v>
+      </c>
+      <c r="AC9" s="30">
+        <v>2</v>
+      </c>
+      <c r="AD9" s="31"/>
+      <c r="AE9" s="9">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A10" s="33">
+      <c r="A10" s="22">
         <v>108</v>
       </c>
-      <c r="B10" s="17"/>
+      <c r="B10" s="25"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="10">
-        <v>2</v>
-      </c>
-      <c r="F10" s="10">
-        <v>2</v>
-      </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="10">
-        <v>2</v>
-      </c>
-      <c r="K10" s="10">
-        <v>2</v>
-      </c>
-      <c r="L10" s="10">
-        <v>2</v>
-      </c>
-      <c r="M10" s="10">
-        <v>2</v>
-      </c>
-      <c r="N10" s="10">
-        <v>2</v>
-      </c>
-      <c r="O10" s="12">
-        <v>2</v>
-      </c>
-      <c r="P10" s="10">
-        <v>2</v>
-      </c>
-      <c r="Q10" s="10">
-        <v>2</v>
-      </c>
-      <c r="R10" s="10">
-        <v>2</v>
-      </c>
-      <c r="S10" s="10">
-        <v>2</v>
-      </c>
-      <c r="T10" s="12">
-        <v>2</v>
-      </c>
-      <c r="U10" s="12">
-        <v>2</v>
-      </c>
-      <c r="V10" s="10">
-        <v>2</v>
-      </c>
-      <c r="W10" s="10">
-        <v>2</v>
-      </c>
-      <c r="X10" s="12">
-        <v>2</v>
-      </c>
-      <c r="Y10" s="12">
-        <v>2</v>
-      </c>
-      <c r="Z10" s="12">
-        <v>2</v>
-      </c>
-      <c r="AA10" s="12">
-        <v>2</v>
-      </c>
-      <c r="AB10" s="12">
-        <v>2</v>
-      </c>
-      <c r="AC10" s="21"/>
-      <c r="AD10" s="22"/>
-      <c r="AE10" s="10">
+      <c r="D10" s="29"/>
+      <c r="E10" s="9">
+        <v>2</v>
+      </c>
+      <c r="F10" s="9">
+        <v>2</v>
+      </c>
+      <c r="G10" s="15"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="9">
+        <v>2</v>
+      </c>
+      <c r="K10" s="9">
+        <v>2</v>
+      </c>
+      <c r="L10" s="9">
+        <v>2</v>
+      </c>
+      <c r="M10" s="9">
+        <v>2</v>
+      </c>
+      <c r="N10" s="9">
+        <v>2</v>
+      </c>
+      <c r="O10" s="10">
+        <v>2</v>
+      </c>
+      <c r="P10" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q10" s="9">
+        <v>2</v>
+      </c>
+      <c r="R10" s="9">
+        <v>2</v>
+      </c>
+      <c r="S10" s="9">
+        <v>2</v>
+      </c>
+      <c r="T10" s="10">
+        <v>2</v>
+      </c>
+      <c r="U10" s="10">
+        <v>2</v>
+      </c>
+      <c r="V10" s="9">
+        <v>2</v>
+      </c>
+      <c r="W10" s="9">
+        <v>2</v>
+      </c>
+      <c r="X10" s="10">
+        <v>2</v>
+      </c>
+      <c r="Y10" s="10">
+        <v>2</v>
+      </c>
+      <c r="Z10" s="10">
+        <v>2</v>
+      </c>
+      <c r="AA10" s="10">
+        <v>2</v>
+      </c>
+      <c r="AB10" s="10">
+        <v>2</v>
+      </c>
+      <c r="AC10" s="32"/>
+      <c r="AD10" s="33"/>
+      <c r="AE10" s="9">
         <v>2</v>
       </c>
     </row>
@@ -7340,83 +7350,83 @@
       <c r="A11" s="2">
         <v>109</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="9">
         <v>10</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="E11" s="10">
+      <c r="E11" s="9">
         <v>10</v>
       </c>
-      <c r="F11" s="10">
+      <c r="F11" s="9">
         <v>10</v>
       </c>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="10">
+      <c r="G11" s="15"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="9">
         <v>10</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="9">
         <v>10</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="9">
         <v>10</v>
       </c>
-      <c r="M11" s="10">
+      <c r="M11" s="9">
         <v>10</v>
       </c>
-      <c r="N11" s="10">
+      <c r="N11" s="9">
         <v>10</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="10">
         <v>10</v>
       </c>
-      <c r="P11" s="10">
+      <c r="P11" s="9">
         <v>10</v>
       </c>
-      <c r="Q11" s="10">
+      <c r="Q11" s="9">
         <v>10</v>
       </c>
-      <c r="R11" s="10">
+      <c r="R11" s="9">
         <v>10</v>
       </c>
-      <c r="S11" s="10">
+      <c r="S11" s="9">
         <v>10</v>
       </c>
-      <c r="T11" s="10">
+      <c r="T11" s="9">
         <v>10</v>
       </c>
-      <c r="U11" s="10">
+      <c r="U11" s="9">
         <v>10</v>
       </c>
-      <c r="V11" s="10">
+      <c r="V11" s="9">
         <v>10</v>
       </c>
-      <c r="W11" s="10">
+      <c r="W11" s="9">
         <v>10</v>
       </c>
-      <c r="X11" s="10">
+      <c r="X11" s="9">
         <v>10</v>
       </c>
-      <c r="Y11" s="10">
+      <c r="Y11" s="9">
         <v>10</v>
       </c>
-      <c r="Z11" s="10">
+      <c r="Z11" s="9">
         <v>10</v>
       </c>
-      <c r="AA11" s="10">
+      <c r="AA11" s="9">
         <v>10</v>
       </c>
-      <c r="AB11" s="10">
+      <c r="AB11" s="9">
         <v>10</v>
       </c>
-      <c r="AC11" s="10">
+      <c r="AC11" s="9">
         <v>10</v>
       </c>
-      <c r="AD11" s="10">
+      <c r="AD11" s="9">
         <v>10</v>
       </c>
-      <c r="AE11" s="10">
+      <c r="AE11" s="9">
         <v>10</v>
       </c>
     </row>
@@ -7424,83 +7434,83 @@
       <c r="A12" s="2">
         <v>110</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="9">
         <v>5</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="E12" s="12">
+      <c r="E12" s="10">
         <v>5</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="10">
         <v>5</v>
       </c>
-      <c r="G12" s="26"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="10">
+      <c r="G12" s="15"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="9">
         <v>5</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="9">
         <v>5</v>
       </c>
-      <c r="L12" s="12">
+      <c r="L12" s="10">
         <v>5</v>
       </c>
-      <c r="M12" s="12">
+      <c r="M12" s="10">
         <v>5</v>
       </c>
-      <c r="N12" s="10">
+      <c r="N12" s="9">
         <v>5</v>
       </c>
-      <c r="O12" s="12">
+      <c r="O12" s="10">
         <v>5</v>
       </c>
-      <c r="P12" s="10">
+      <c r="P12" s="9">
         <v>5</v>
       </c>
-      <c r="Q12" s="10">
+      <c r="Q12" s="9">
         <v>5</v>
       </c>
-      <c r="R12" s="10">
+      <c r="R12" s="9">
         <v>5</v>
       </c>
-      <c r="S12" s="10">
+      <c r="S12" s="9">
         <v>5</v>
       </c>
-      <c r="T12" s="10">
+      <c r="T12" s="9">
         <v>5</v>
       </c>
-      <c r="U12" s="10">
+      <c r="U12" s="9">
         <v>5</v>
       </c>
-      <c r="V12" s="10">
+      <c r="V12" s="9">
         <v>5</v>
       </c>
-      <c r="W12" s="10">
+      <c r="W12" s="9">
         <v>5</v>
       </c>
-      <c r="X12" s="10">
+      <c r="X12" s="9">
         <v>5</v>
       </c>
-      <c r="Y12" s="10">
+      <c r="Y12" s="9">
         <v>5</v>
       </c>
-      <c r="Z12" s="12">
+      <c r="Z12" s="10">
         <v>5</v>
       </c>
-      <c r="AA12" s="10">
+      <c r="AA12" s="9">
         <v>5</v>
       </c>
-      <c r="AB12" s="10">
+      <c r="AB12" s="9">
         <v>5</v>
       </c>
-      <c r="AC12" s="10">
+      <c r="AC12" s="9">
         <v>5</v>
       </c>
-      <c r="AD12" s="10">
+      <c r="AD12" s="9">
         <v>5</v>
       </c>
-      <c r="AE12" s="10">
+      <c r="AE12" s="9">
         <v>5</v>
       </c>
     </row>
@@ -7518,16 +7528,16 @@
       <c r="F13" s="7">
         <v>4</v>
       </c>
-      <c r="G13" s="26"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="28"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="17"/>
       <c r="J13" s="7">
         <v>4</v>
       </c>
       <c r="K13" s="7">
         <v>4</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="26">
         <v>4</v>
       </c>
       <c r="M13" s="7">
@@ -7539,7 +7549,7 @@
       <c r="O13" s="7">
         <v>4</v>
       </c>
-      <c r="P13" s="9">
+      <c r="P13" s="26">
         <v>4</v>
       </c>
       <c r="Q13" s="7">
@@ -7602,16 +7612,16 @@
       <c r="F14" s="7">
         <v>4</v>
       </c>
-      <c r="G14" s="26"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="28"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="17"/>
       <c r="J14" s="7">
         <v>4</v>
       </c>
       <c r="K14" s="7">
         <v>4</v>
       </c>
-      <c r="L14" s="13"/>
+      <c r="L14" s="27"/>
       <c r="M14" s="7">
         <v>4</v>
       </c>
@@ -7621,7 +7631,7 @@
       <c r="O14" s="7">
         <v>4</v>
       </c>
-      <c r="P14" s="13"/>
+      <c r="P14" s="27"/>
       <c r="Q14" s="7">
         <v>4</v>
       </c>
@@ -7672,27 +7682,29 @@
       <c r="A15" s="2">
         <v>203</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="26">
         <v>4</v>
       </c>
       <c r="C15" s="2"/>
-      <c r="D15" s="14"/>
+      <c r="D15" s="11">
+        <v>4</v>
+      </c>
       <c r="E15" s="6">
         <v>4</v>
       </c>
       <c r="F15" s="6">
         <v>4</v>
       </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="28"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="17"/>
       <c r="J15" s="7">
         <v>4</v>
       </c>
       <c r="K15" s="7">
         <v>4</v>
       </c>
-      <c r="L15" s="13"/>
+      <c r="L15" s="27"/>
       <c r="M15" s="7">
         <v>4</v>
       </c>
@@ -7702,7 +7714,7 @@
       <c r="O15" s="7">
         <v>4</v>
       </c>
-      <c r="P15" s="11"/>
+      <c r="P15" s="28"/>
       <c r="Q15" s="7">
         <v>4</v>
       </c>
@@ -7753,7 +7765,7 @@
       <c r="A16" s="2">
         <v>204</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="28"/>
       <c r="C16" s="2"/>
       <c r="E16" s="7">
         <v>4</v>
@@ -7761,16 +7773,16 @@
       <c r="F16" s="6">
         <v>4</v>
       </c>
-      <c r="G16" s="26"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="28"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="17"/>
       <c r="J16" s="7">
         <v>4</v>
       </c>
       <c r="K16" s="7">
         <v>4</v>
       </c>
-      <c r="L16" s="13"/>
+      <c r="L16" s="27"/>
       <c r="M16" s="7">
         <v>4</v>
       </c>
@@ -7801,10 +7813,10 @@
       <c r="V16" s="7">
         <v>4</v>
       </c>
-      <c r="W16" s="9">
-        <v>4</v>
-      </c>
-      <c r="X16" s="9">
+      <c r="W16" s="26">
+        <v>4</v>
+      </c>
+      <c r="X16" s="26">
         <v>4</v>
       </c>
       <c r="Y16" s="7">
@@ -7843,16 +7855,16 @@
       <c r="F17" s="7">
         <v>4</v>
       </c>
-      <c r="G17" s="26"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="28"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="17"/>
       <c r="J17" s="7">
         <v>4</v>
       </c>
       <c r="K17" s="7">
         <v>4</v>
       </c>
-      <c r="L17" s="13"/>
+      <c r="L17" s="27"/>
       <c r="M17" s="7">
         <v>4</v>
       </c>
@@ -7883,8 +7895,8 @@
       <c r="V17" s="6">
         <v>4</v>
       </c>
-      <c r="W17" s="11"/>
-      <c r="X17" s="11"/>
+      <c r="W17" s="28"/>
+      <c r="X17" s="28"/>
       <c r="Y17" s="7">
         <v>4</v>
       </c>
@@ -7911,7 +7923,7 @@
       <c r="A18" s="2">
         <v>206</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="26">
         <v>4</v>
       </c>
       <c r="C18" s="2"/>
@@ -7921,16 +7933,16 @@
       <c r="F18" s="7">
         <v>4</v>
       </c>
-      <c r="G18" s="26"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="28"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="17"/>
       <c r="J18" s="7">
         <v>4</v>
       </c>
       <c r="K18" s="7">
         <v>4</v>
       </c>
-      <c r="L18" s="11"/>
+      <c r="L18" s="28"/>
       <c r="M18" s="6">
         <v>4</v>
       </c>
@@ -7949,13 +7961,13 @@
       <c r="R18" s="7">
         <v>4</v>
       </c>
-      <c r="S18" s="9">
+      <c r="S18" s="26">
         <v>4</v>
       </c>
       <c r="T18" s="7">
         <v>4</v>
       </c>
-      <c r="U18" s="9">
+      <c r="U18" s="26">
         <v>4</v>
       </c>
       <c r="V18" s="7">
@@ -7993,7 +8005,7 @@
       <c r="A19" s="2">
         <v>207</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="28"/>
       <c r="C19" s="2"/>
       <c r="E19" s="7">
         <v>4</v>
@@ -8001,9 +8013,9 @@
       <c r="F19" s="7">
         <v>4</v>
       </c>
-      <c r="G19" s="26"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="17"/>
       <c r="J19" s="7">
         <v>4</v>
       </c>
@@ -8022,7 +8034,7 @@
       <c r="O19" s="7">
         <v>4</v>
       </c>
-      <c r="P19" s="9">
+      <c r="P19" s="26">
         <v>4</v>
       </c>
       <c r="Q19" s="7">
@@ -8031,15 +8043,15 @@
       <c r="R19" s="7">
         <v>4</v>
       </c>
-      <c r="S19" s="13"/>
+      <c r="S19" s="27"/>
       <c r="T19" s="7">
         <v>4</v>
       </c>
-      <c r="U19" s="11"/>
-      <c r="V19" s="19">
-        <v>4</v>
-      </c>
-      <c r="W19" s="20"/>
+      <c r="U19" s="28"/>
+      <c r="V19" s="30">
+        <v>4</v>
+      </c>
+      <c r="W19" s="31"/>
       <c r="X19" s="7">
         <v>4</v>
       </c>
@@ -8069,75 +8081,75 @@
       <c r="A20" s="2">
         <v>208</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="10">
         <v>4</v>
       </c>
       <c r="C20" s="2"/>
-      <c r="E20" s="10">
-        <v>4</v>
-      </c>
-      <c r="F20" s="10">
-        <v>4</v>
-      </c>
-      <c r="G20" s="29"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="10">
-        <v>4</v>
-      </c>
-      <c r="K20" s="10">
-        <v>4</v>
-      </c>
-      <c r="L20" s="10">
-        <v>4</v>
-      </c>
-      <c r="M20" s="10">
-        <v>4</v>
-      </c>
-      <c r="N20" s="10">
-        <v>4</v>
-      </c>
-      <c r="O20" s="10">
-        <v>4</v>
-      </c>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="10">
-        <v>4</v>
-      </c>
-      <c r="R20" s="10">
-        <v>4</v>
-      </c>
-      <c r="S20" s="11"/>
-      <c r="T20" s="10">
-        <v>4</v>
-      </c>
-      <c r="U20" s="10">
-        <v>4</v>
-      </c>
-      <c r="V20" s="21"/>
-      <c r="W20" s="22"/>
-      <c r="X20" s="10">
-        <v>4</v>
-      </c>
-      <c r="Y20" s="10">
-        <v>4</v>
-      </c>
-      <c r="Z20" s="10">
-        <v>4</v>
-      </c>
-      <c r="AA20" s="10">
-        <v>4</v>
-      </c>
-      <c r="AB20" s="10">
-        <v>4</v>
-      </c>
-      <c r="AC20" s="12">
-        <v>4</v>
-      </c>
-      <c r="AD20" s="10">
-        <v>4</v>
-      </c>
-      <c r="AE20" s="10">
+      <c r="E20" s="9">
+        <v>4</v>
+      </c>
+      <c r="F20" s="9">
+        <v>4</v>
+      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="9">
+        <v>4</v>
+      </c>
+      <c r="K20" s="9">
+        <v>4</v>
+      </c>
+      <c r="L20" s="9">
+        <v>4</v>
+      </c>
+      <c r="M20" s="9">
+        <v>4</v>
+      </c>
+      <c r="N20" s="9">
+        <v>4</v>
+      </c>
+      <c r="O20" s="9">
+        <v>4</v>
+      </c>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="9">
+        <v>4</v>
+      </c>
+      <c r="R20" s="9">
+        <v>4</v>
+      </c>
+      <c r="S20" s="28"/>
+      <c r="T20" s="9">
+        <v>4</v>
+      </c>
+      <c r="U20" s="9">
+        <v>4</v>
+      </c>
+      <c r="V20" s="32"/>
+      <c r="W20" s="33"/>
+      <c r="X20" s="9">
+        <v>4</v>
+      </c>
+      <c r="Y20" s="9">
+        <v>4</v>
+      </c>
+      <c r="Z20" s="9">
+        <v>4</v>
+      </c>
+      <c r="AA20" s="9">
+        <v>4</v>
+      </c>
+      <c r="AB20" s="9">
+        <v>4</v>
+      </c>
+      <c r="AC20" s="10">
+        <v>4</v>
+      </c>
+      <c r="AD20" s="9">
+        <v>4</v>
+      </c>
+      <c r="AE20" s="9">
         <v>4</v>
       </c>
     </row>
@@ -8150,16 +8162,16 @@
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="S18:S20"/>
     <mergeCell ref="U18:U19"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="AC4:AC5"/>
     <mergeCell ref="P13:P15"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="V9:W9"/>
     <mergeCell ref="AC9:AD10"/>
     <mergeCell ref="L13:L18"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="AC4:AC5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>